<commit_message>
Updates on effective density and mobility
Curve fitting on effective density data added. All mobility size distribution data compiled, averaged and visualized.
</commit_message>
<xml_diff>
--- a/inputs/odias_labels_new.xlsx
+++ b/inputs/odias_labels_new.xlsx
@@ -1,32 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\hmdni\OneDrive\Documents\GitHub\odias\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A96DDCF-AAE1-4FEA-AB95-787ED5029D87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9337714F-7E36-412B-A716-D13081D21F92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="07FEB25_EXCOLAPS_TANDEM" sheetId="17" r:id="rId1"/>
-    <sheet name="06FEB25_R2_EXAGGLOM_TANDEM" sheetId="16" r:id="rId2"/>
-    <sheet name="06FEB25_R1_EXAGGLOM_TANDEM" sheetId="15" r:id="rId3"/>
-    <sheet name="30JUL24_HIGHAGGLOM_TANDEM" sheetId="14" r:id="rId4"/>
-    <sheet name="26JUL24_LOWAGGLOM_TANDEM" sheetId="13" r:id="rId5"/>
-    <sheet name="28AUG24_HIGHAGGLOM_TANDEM" sheetId="12" r:id="rId6"/>
-    <sheet name="20AUG24_HIGHAGGLOM_TANDEM" sheetId="11" r:id="rId7"/>
-    <sheet name="20AUG24_LOWAGGLOM_TANDEM" sheetId="10" r:id="rId8"/>
-    <sheet name="21AUG24_HIGHAGGLOM_TANDEM" sheetId="9" r:id="rId9"/>
-    <sheet name="19AUG24_LOWAGGLOM_TANDEM" sheetId="8" r:id="rId10"/>
-    <sheet name="ET017_NIT013_AIR16_DIST" sheetId="7" r:id="rId11"/>
-    <sheet name="23JUL24_SWEEP_ON_AIR" sheetId="5" r:id="rId12"/>
-    <sheet name="20JUL24_SWEEP_ON_NITROGEN" sheetId="6" r:id="rId13"/>
-    <sheet name="13SEP24_SWEEP_ON_FUEL" sheetId="4" r:id="rId14"/>
+    <sheet name="MOBIL_DIST_FEB25" sheetId="22" r:id="rId1"/>
+    <sheet name="12FEB25_R2_EXAGLOM_TANDEM" sheetId="21" r:id="rId2"/>
+    <sheet name="12FEB25_R1_EXAGLOM_TANDEM" sheetId="20" r:id="rId3"/>
+    <sheet name="11FEB25_LOAGLOM_TANDEM" sheetId="19" r:id="rId4"/>
+    <sheet name="08FEB25_EXCOLAPS_TANDEM" sheetId="18" r:id="rId5"/>
+    <sheet name="07FEB25_EXCOLAPS_TANDEM" sheetId="17" r:id="rId6"/>
+    <sheet name="06FEB25_R2_EXAGGLOM_TANDEM" sheetId="16" r:id="rId7"/>
+    <sheet name="06FEB25_R1_EXAGGLOM_TANDEM" sheetId="15" r:id="rId8"/>
+    <sheet name="30JUL24_HIGHAGGLOM_TANDEM" sheetId="14" r:id="rId9"/>
+    <sheet name="26JUL24_LOWAGGLOM_TANDEM" sheetId="13" r:id="rId10"/>
+    <sheet name="28AUG24_HIGHAGGLOM_TANDEM" sheetId="12" r:id="rId11"/>
+    <sheet name="20AUG24_HIGHAGGLOM_TANDEM" sheetId="11" r:id="rId12"/>
+    <sheet name="20AUG24_LOWAGGLOM_TANDEM" sheetId="10" r:id="rId13"/>
+    <sheet name="21AUG24_HIGHAGGLOM_TANDEM" sheetId="9" r:id="rId14"/>
+    <sheet name="19AUG24_LOWAGGLOM_TANDEM" sheetId="8" r:id="rId15"/>
+    <sheet name="ET017_NIT013_AIR16_DIST" sheetId="7" r:id="rId16"/>
+    <sheet name="23JUL24_SWEEP_ON_AIR" sheetId="5" r:id="rId17"/>
+    <sheet name="20JUL24_SWEEP_ON_NITROGEN" sheetId="6" r:id="rId18"/>
+    <sheet name="13SEP24_SWEEP_ON_FUEL" sheetId="4" r:id="rId19"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="44">
   <si>
     <t>Q_f</t>
   </si>
@@ -148,6 +153,39 @@
   </si>
   <si>
     <t>07 FEB. 25</t>
+  </si>
+  <si>
+    <t>08 FEB. 25</t>
+  </si>
+  <si>
+    <t>AGLOM</t>
+  </si>
+  <si>
+    <t>11 FEB. 25</t>
+  </si>
+  <si>
+    <t>12 FEB. 25</t>
+  </si>
+  <si>
+    <t>Aglom</t>
+  </si>
+  <si>
+    <t>Lo-Aglom</t>
+  </si>
+  <si>
+    <t>Mod-Colaps</t>
+  </si>
+  <si>
+    <t>Hi-Aglom</t>
+  </si>
+  <si>
+    <t>Ex-Colaps</t>
+  </si>
+  <si>
+    <t>Condition</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
@@ -172,12 +210,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -192,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -200,6 +250,11 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -479,7 +534,301 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2AE00AE-0F5D-489D-A932-FE925984278A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9472C2C5-74CD-455E-BDBC-C60A45D7448D}">
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="B15" s="9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E795ADCB-0CBC-4EFE-B830-C148C8037C17}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>46.9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>64.400000000000006</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>75.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7">
+        <v>88.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8">
+        <v>103.7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9">
+        <v>121.6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>142.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>195.8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>229.4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="C14" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAD73EBE-1EAA-44DC-A0C0-8157A532E2E4}">
   <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -491,7 +840,7 @@
         <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>27</v>
@@ -499,151 +848,686 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C2" s="3">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C3" s="3">
-        <v>88.7</v>
+        <v>46.9</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C4" s="3">
-        <v>98.4</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C5" s="3">
-        <v>109.1</v>
+        <v>64.400000000000006</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C6" s="3">
-        <v>120.9</v>
+        <v>75.5</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C7" s="3">
-        <v>134.11108308881299</v>
+        <v>88.5</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C8" s="3">
-        <v>148.69999999999999</v>
+        <v>103.7</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C9" s="3">
-        <v>164.9</v>
+        <v>121.6</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C10" s="3">
-        <v>182.8</v>
+        <v>142.5</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C11" s="3">
-        <v>202.8</v>
+        <v>167</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="4">
-        <v>224.8</v>
+        <v>4</v>
+      </c>
+      <c r="C12" s="3">
+        <v>195.8</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13">
-        <v>249.3</v>
+        <v>4</v>
+      </c>
+      <c r="C13" s="3">
+        <v>229.4</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="C14" s="1" t="s">
+      <c r="A14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="3">
+        <v>268.89999999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C15" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44632B00-FC5D-4DBD-8F00-AB03E4F5356D}">
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="3">
+        <v>46.9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="3">
+        <v>64.400000000000006</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="3">
+        <v>75.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="3">
+        <v>88.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="3">
+        <v>103.7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="3">
+        <v>121.6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="3">
+        <v>142.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="3">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="3">
+        <v>195.8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="3">
+        <v>229.4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="3">
+        <v>291.2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C15" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F2C525F-95DB-48C6-90C1-5B53F4E14E89}">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2">
+        <v>29.130528992918819</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="2">
+        <v>34.135335939708469</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="2">
+        <v>46.9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="2">
+        <v>64.400000000000006</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="2">
+        <v>75.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="2">
+        <v>88.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="2">
+        <v>103.7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="2">
+        <v>121.6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" s="2">
+        <v>142.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" s="2">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="2">
+        <v>195.8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="2">
+        <v>229.4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C16" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41BFA0A0-46FE-44C4-8DCF-97D89F82D692}">
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2">
+        <v>43.3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2">
+        <v>50.8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2">
+        <v>59.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2">
+        <v>69.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2">
+        <v>81.7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="2">
+        <v>95.8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="2">
+        <v>112.3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="2">
+        <v>131.6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="2">
+        <v>154.30000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="2">
+        <v>180.8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="2">
+        <v>211.9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="2">
+        <v>248.4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="2">
+        <v>291.2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="C15" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{389217E3-4E52-4BC7-B8D7-4BC23C109860}">
   <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -816,7 +1700,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FCC4001-51B9-4279-A3FF-BA4CAE7D4664}">
   <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1053,7 +1937,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2025863E-BC07-424F-B878-D13AF188D89A}">
   <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1365,7 +2249,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD54F46B-74D1-410F-8672-1CA20743FEB6}">
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1523,7 +2407,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FBEF317-768D-4A04-98BA-90E8FE55E3DF}">
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1661,6 +2545,813 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E0260B3-3DBF-467C-9F72-187D3B479951}">
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="3">
+        <v>63.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="3">
+        <v>71.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="3">
+        <v>80.8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="3">
+        <v>102.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="3">
+        <v>115.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="3">
+        <v>146.4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="3">
+        <v>164.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="3">
+        <v>185.7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="3">
+        <v>209.2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="3">
+        <v>235.6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="3">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="C15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C96F583-DB7F-42CC-82A6-033A7076AFF0}">
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="3">
+        <v>67.599999999999994</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="3">
+        <v>76.099999999999994</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="3">
+        <v>85.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="3">
+        <v>96.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="3">
+        <v>108.7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="3">
+        <v>122.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="3">
+        <v>137.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="3">
+        <v>155.4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="3">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12">
+        <v>197.1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="C14" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CF807E3-9513-422E-92EA-744FA87D082B}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="3">
+        <v>30.8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="3">
+        <v>46.8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="3">
+        <v>57.8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="3">
+        <v>71.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="3">
+        <v>87.8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="3">
+        <v>108.2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="3">
+        <v>133.4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="3">
+        <v>164.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>202.8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B99EF233-E62F-473B-94D2-E2A467303827}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="3">
+        <v>93.4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="3">
+        <v>103.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="3">
+        <v>114.9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="3">
+        <v>127.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="3">
+        <v>141.19999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="3">
+        <v>156.6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="3">
+        <v>173.6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="3">
+        <v>192.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="3">
+        <v>213.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="3">
+        <v>236.7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1"/>
+      <c r="C12" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2AE00AE-0F5D-489D-A932-FE925984278A}">
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="3">
+        <v>88.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="3">
+        <v>98.4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="3">
+        <v>109.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="3">
+        <v>120.9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="3">
+        <v>134.11108308881299</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="3">
+        <v>148.69999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="3">
+        <v>164.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="3">
+        <v>182.8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="3">
+        <v>202.8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="4">
+        <v>224.8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13">
+        <v>249.3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="C14" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{430790D4-4E38-4D50-85D3-BBBD044276D2}">
   <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1809,7 +3500,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98B65913-8716-4830-8572-CA5A30057124}">
   <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1958,7 +3649,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56594976-E9EE-43CC-9355-D71CEE81843A}">
   <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2129,866 +3820,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E795ADCB-0CBC-4EFE-B830-C148C8037C17}">
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3">
-        <v>46.9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5">
-        <v>64.400000000000006</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6">
-        <v>75.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7">
-        <v>88.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8">
-        <v>103.7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9">
-        <v>121.6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" t="s">
-        <v>3</v>
-      </c>
-      <c r="C10">
-        <v>142.5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" t="s">
-        <v>3</v>
-      </c>
-      <c r="C11">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" t="s">
-        <v>3</v>
-      </c>
-      <c r="C12">
-        <v>195.8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>3</v>
-      </c>
-      <c r="C13">
-        <v>229.4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="C14" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAD73EBE-1EAA-44DC-A0C0-8157A532E2E4}">
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="3">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="3">
-        <v>46.9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="3">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="3">
-        <v>64.400000000000006</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="3">
-        <v>75.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="3">
-        <v>88.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="3">
-        <v>103.7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="3">
-        <v>121.6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="3">
-        <v>142.5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" s="3">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12" s="3">
-        <v>195.8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" s="3">
-        <v>229.4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" s="3">
-        <v>268.89999999999998</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C15" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44632B00-FC5D-4DBD-8F00-AB03E4F5356D}">
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="3">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="3">
-        <v>46.9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="3">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="3">
-        <v>64.400000000000006</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="3">
-        <v>75.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="3">
-        <v>88.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="3">
-        <v>103.7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="3">
-        <v>121.6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="3">
-        <v>142.5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" s="3">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12" s="3">
-        <v>195.8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" s="3">
-        <v>229.4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" s="3">
-        <v>291.2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C15" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F2C525F-95DB-48C6-90C1-5B53F4E14E89}">
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="2">
-        <v>29.130528992918819</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="2">
-        <v>34.135335939708469</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="2">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="2">
-        <v>46.9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="2">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" s="2">
-        <v>64.400000000000006</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" s="2">
-        <v>75.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="2">
-        <v>88.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" t="s">
-        <v>3</v>
-      </c>
-      <c r="C10" s="2">
-        <v>103.7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>3</v>
-      </c>
-      <c r="C11" s="2">
-        <v>121.6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" t="s">
-        <v>3</v>
-      </c>
-      <c r="C12" s="2">
-        <v>142.5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" t="s">
-        <v>3</v>
-      </c>
-      <c r="C13" s="2">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C14" s="2">
-        <v>195.8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" t="s">
-        <v>3</v>
-      </c>
-      <c r="C15" s="2">
-        <v>229.4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C16" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41BFA0A0-46FE-44C4-8DCF-97D89F82D692}">
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2">
-        <v>43.3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="2">
-        <v>50.8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="2">
-        <v>59.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="2">
-        <v>69.7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="2">
-        <v>81.7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="2">
-        <v>95.8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="2">
-        <v>112.3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="2">
-        <v>131.6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="2">
-        <v>154.30000000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" s="2">
-        <v>180.8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12" s="2">
-        <v>211.9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" s="2">
-        <v>248.4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" s="2">
-        <v>291.2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-      <c r="C15" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>